<commit_message>
Use gender-neutral language (fiance/they) instead of groom/he, keeping Bride terminology as-is
</commit_message>
<xml_diff>
--- a/Newlywed Answer Form.xlsx
+++ b/Newlywed Answer Form.xlsx
@@ -515,14 +515,14 @@
     <row r="5" ht="34" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2.  Send this file to the fiancé and ask him to fill in ONLY the Answer column.</t>
+          <t>2.  Send this file to the fiancé and ask them to fill in ONLY the Answer column.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="34" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>3.  Once he sends it back, re-upload this exact file into the Bachelorette Newlywed Game app to auto-build the game board.</t>
+          <t>3.  Once you get it back, re-upload this exact file into the Bachelorette Newlywed Game app to auto-build the game board.</t>
         </is>
       </c>
     </row>

</xml_diff>